<commit_message>
test: reconcile Sprint 5 deployment security workbook
</commit_message>
<xml_diff>
--- a/docs/testing/sprint-5-security-permission-test-cases.xlsx
+++ b/docs/testing/sprint-5-security-permission-test-cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\08_Personals\School Portfolio\GradNavi\docs\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0339D9E5-8273-4061-8C54-D2F943770102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D90725E-4DD9-465E-BBB7-464E89EFBBC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1313" uniqueCount="536">
   <si>
     <t>GradNavi WBS 8.3 Security and Permission Test Tracker</t>
   </si>
@@ -1626,6 +1626,24 @@
   </si>
   <si>
     <t>Local WBS 8.3 security execution complete: 30 Pass, 0 Blocked, 2 Deferred deployment reviews. S5-SEC-FE-01 passed after WBS 7.7 integration.</t>
+  </si>
+  <si>
+    <t>Pass (project-lead reported)</t>
+  </si>
+  <si>
+    <t>Post-deployment security check reported PASS by project lead. Detailed configuration evidence has not been independently reviewed.</t>
+  </si>
+  <si>
+    <t>Follow-up reported 13 October 2026. Original status: Deferred. Actual executor, execution date and supporting configuration evidence require confirmation.</t>
+  </si>
+  <si>
+    <t>Reported Pass</t>
+  </si>
+  <si>
+    <t>Project lead confirmed PASS following deployment. Independent configuration evidence not supplied.</t>
+  </si>
+  <si>
+    <t>Reported 13 October 2026. Original evidence state: Deferred. Evidence location and actual execution details pending.</t>
   </si>
 </sst>
 </file>
@@ -4791,7 +4809,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="32" spans="1:22" ht="57">
+    <row r="32" spans="1:22" ht="71.25">
       <c r="A32" s="6" t="s">
         <v>378</v>
       </c>
@@ -4826,13 +4844,14 @@
         <v>215</v>
       </c>
       <c r="L32" s="6" t="s">
-        <v>20</v>
+        <v>530</v>
       </c>
       <c r="M32" s="6"/>
-      <c r="N32" s="6"/>
-      <c r="O32" s="6" t="str">
-        <f>IF(OR(K32="Fail",L32="Fail"),"Fail",IF(L32="Blocked","Blocked",IF(L32="Deferred","Deferred",IF(AND(OR(K32="Pass",K32="N/A"),OR(L32="Pass",L32="N/A")),"Pass","Not Run"))))</f>
-        <v>Deferred</v>
+      <c r="N32" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="O32" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="P32" s="6"/>
       <c r="Q32" s="7"/>
@@ -4841,12 +4860,14 @@
       <c r="T32" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="U32" s="6"/>
+      <c r="U32" s="6" t="s">
+        <v>532</v>
+      </c>
       <c r="V32" s="6" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="33" spans="1:22" ht="57">
+    <row r="33" spans="1:22" ht="71.25">
       <c r="A33" s="6" t="s">
         <v>386</v>
       </c>
@@ -4881,13 +4902,14 @@
         <v>215</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>20</v>
+        <v>530</v>
       </c>
       <c r="M33" s="6"/>
-      <c r="N33" s="6"/>
-      <c r="O33" s="6" t="str">
-        <f>IF(OR(K33="Fail",L33="Fail"),"Fail",IF(L33="Blocked","Blocked",IF(L33="Deferred","Deferred",IF(AND(OR(K33="Pass",K33="N/A"),OR(L33="Pass",L33="N/A")),"Pass","Not Run"))))</f>
-        <v>Deferred</v>
+      <c r="N33" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="O33" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="P33" s="6"/>
       <c r="Q33" s="7"/>
@@ -4896,7 +4918,9 @@
       <c r="T33" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="U33" s="6"/>
+      <c r="U33" s="6" t="s">
+        <v>532</v>
+      </c>
       <c r="V33" s="6" t="s">
         <v>390</v>
       </c>
@@ -6944,7 +6968,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="28.5">
+    <row r="59" spans="1:11" ht="42.75">
       <c r="A59" s="6" t="s">
         <v>502</v>
       </c>
@@ -6958,18 +6982,22 @@
         <v>402</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>20</v>
+        <v>533</v>
       </c>
       <c r="F59" s="6"/>
-      <c r="G59" s="6"/>
+      <c r="G59" s="6" t="s">
+        <v>534</v>
+      </c>
       <c r="H59" s="6" t="s">
         <v>501</v>
       </c>
       <c r="I59" s="6"/>
       <c r="J59" s="7"/>
-      <c r="K59" s="6"/>
-    </row>
-    <row r="60" spans="1:11" ht="28.5">
+      <c r="K59" s="6" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="42.75">
       <c r="A60" s="6" t="s">
         <v>504</v>
       </c>
@@ -6983,16 +7011,20 @@
         <v>402</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>20</v>
+        <v>533</v>
       </c>
       <c r="F60" s="6"/>
-      <c r="G60" s="6"/>
+      <c r="G60" s="6" t="s">
+        <v>534</v>
+      </c>
       <c r="H60" s="6" t="s">
         <v>501</v>
       </c>
       <c r="I60" s="6"/>
       <c r="J60" s="7"/>
-      <c r="K60" s="6"/>
+      <c r="K60" s="6" t="s">
+        <v>535</v>
+      </c>
     </row>
     <row r="61" spans="1:11" ht="71.25">
       <c r="A61" t="s">

</xml_diff>

<commit_message>
test(sprint5): reconcile deployment security evidence in workbook
</commit_message>
<xml_diff>
--- a/docs/testing/sprint-5-security-permission-test-cases.xlsx
+++ b/docs/testing/sprint-5-security-permission-test-cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\08_Personals\School Portfolio\GradNavi\docs\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D90725E-4DD9-465E-BBB7-464E89EFBBC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7785C65D-DEF6-40C9-AD06-7EE61FC423FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1313" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1317" uniqueCount="538">
   <si>
     <t>GradNavi WBS 8.3 Security and Permission Test Tracker</t>
   </si>
@@ -1628,15 +1628,9 @@
     <t>Local WBS 8.3 security execution complete: 30 Pass, 0 Blocked, 2 Deferred deployment reviews. S5-SEC-FE-01 passed after WBS 7.7 integration.</t>
   </si>
   <si>
-    <t>Pass (project-lead reported)</t>
-  </si>
-  <si>
     <t>Post-deployment security check reported PASS by project lead. Detailed configuration evidence has not been independently reviewed.</t>
   </si>
   <si>
-    <t>Follow-up reported 13 October 2026. Original status: Deferred. Actual executor, execution date and supporting configuration evidence require confirmation.</t>
-  </si>
-  <si>
     <t>Reported Pass</t>
   </si>
   <si>
@@ -1644,6 +1638,18 @@
   </si>
   <si>
     <t>Reported 13 October 2026. Original evidence state: Deferred. Evidence location and actual execution details pending.</t>
+  </si>
+  <si>
+    <t>docs/testing/evidence/sprint-5/deployment-security/README.md (DEP-01A to DEP-01D)</t>
+  </si>
+  <si>
+    <t>docs/testing/evidence/sprint-5/deployment-security/README.md (DEP-02A to DEP-02B)</t>
+  </si>
+  <si>
+    <t>Additional evidence captured 14 October 2026: Railway variable names reviewed; HTTPS authentication returned 401 with a controlled JSON error; approved CORS origin accepted; unapproved origin rejected. Full production configuration values not independently verified. Screenshots DEP-01A to DEP-01D uploaded to GitHub.</t>
+  </si>
+  <si>
+    <t>Additional evidence captured 14 October 2026: Vercel production API URL confirmed as Railway HTTPS endpoint; authenticated production API request returned 200. Comprehensive browser asset secret-exposure review not independently verified. Screenshots DEP-02A and DEP-02B uploaded to GitHub.</t>
   </si>
 </sst>
 </file>
@@ -2747,7 +2753,7 @@
     <col min="9" max="9" width="28" customWidth="1"/>
     <col min="10" max="10" width="25" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="21" customWidth="1"/>
+    <col min="12" max="12" width="50.75" customWidth="1"/>
     <col min="13" max="13" width="18" customWidth="1"/>
     <col min="14" max="14" width="34" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -4809,7 +4815,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="32" spans="1:22" ht="71.25">
+    <row r="32" spans="1:22" ht="88.5" customHeight="1">
       <c r="A32" s="6" t="s">
         <v>378</v>
       </c>
@@ -4844,30 +4850,34 @@
         <v>215</v>
       </c>
       <c r="L32" s="6" t="s">
-        <v>530</v>
+        <v>12</v>
       </c>
       <c r="M32" s="6"/>
       <c r="N32" s="6" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="O32" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="P32" s="6"/>
+      <c r="P32" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="Q32" s="7"/>
-      <c r="R32" s="6"/>
+      <c r="R32" t="s">
+        <v>534</v>
+      </c>
       <c r="S32" s="6"/>
       <c r="T32" s="6" t="s">
         <v>66</v>
       </c>
       <c r="U32" s="6" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="V32" s="6" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="33" spans="1:22" ht="71.25">
+    <row r="33" spans="1:22" ht="57">
       <c r="A33" s="6" t="s">
         <v>386</v>
       </c>
@@ -4902,24 +4912,28 @@
         <v>215</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>530</v>
+        <v>12</v>
       </c>
       <c r="M33" s="6"/>
       <c r="N33" s="6" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="O33" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="P33" s="6"/>
+      <c r="P33" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="Q33" s="7"/>
-      <c r="R33" s="6"/>
+      <c r="R33" t="s">
+        <v>535</v>
+      </c>
       <c r="S33" s="6"/>
       <c r="T33" s="6" t="s">
         <v>66</v>
       </c>
       <c r="U33" s="6" t="s">
-        <v>532</v>
+        <v>537</v>
       </c>
       <c r="V33" s="6" t="s">
         <v>390</v>
@@ -6982,11 +6996,11 @@
         <v>402</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="F59" s="6"/>
       <c r="G59" s="6" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="H59" s="6" t="s">
         <v>501</v>
@@ -6994,7 +7008,7 @@
       <c r="I59" s="6"/>
       <c r="J59" s="7"/>
       <c r="K59" s="6" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="42.75">
@@ -7011,11 +7025,11 @@
         <v>402</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="F60" s="6"/>
       <c r="G60" s="6" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="H60" s="6" t="s">
         <v>501</v>
@@ -7023,7 +7037,7 @@
       <c r="I60" s="6"/>
       <c r="J60" s="7"/>
       <c r="K60" s="6" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="61" spans="1:11" ht="71.25">

</xml_diff>